<commit_message>
auto-publish commission xlsx: manual
</commit_message>
<xml_diff>
--- a/commission/karin/2026-04.xlsx
+++ b/commission/karin/2026-04.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="April 2026-04" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Invoiced This Month" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="90">
   <si>
     <t>Equine Performance Labs, LLC</t>
   </si>
@@ -149,6 +150,138 @@
   </si>
   <si>
     <t>GRAND TOTAL</t>
+  </si>
+  <si>
+    <t>Invoiced This Month — Karin Williamson — April 2026</t>
+  </si>
+  <si>
+    <t>Every invoice you wrote this month (paid or unpaid). Commission math comes from Tab 1 — this sheet is for visibility only.</t>
+  </si>
+  <si>
+    <t>INV#</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>Vials</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>Commissionable</t>
+  </si>
+  <si>
+    <t>Paid</t>
+  </si>
+  <si>
+    <t>Payment Date</t>
+  </si>
+  <si>
+    <t>Open Bal</t>
+  </si>
+  <si>
+    <t>Promo</t>
+  </si>
+  <si>
+    <t>CASE26</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1048</t>
+  </si>
+  <si>
+    <t>Brazos Valley Equine Hospital-Cypress</t>
+  </si>
+  <si>
+    <t>CASE25</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1052</t>
+  </si>
+  <si>
+    <t>Elgin Equine</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1055</t>
+  </si>
+  <si>
+    <t>Panorama Equine Medical and Surgical Center</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1054</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1061</t>
+  </si>
+  <si>
+    <t>Flying UJ</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>ORD-EPL-1060</t>
+  </si>
+  <si>
+    <t>Equine Athlete Veterinary Services - Simpsonville, KY</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1064</t>
+  </si>
+  <si>
+    <t>Central Washington Equine Hospital</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1063</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1070</t>
+  </si>
+  <si>
+    <t>Outlaw Equine</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1069</t>
+  </si>
+  <si>
+    <t>Double X Veterinary Services</t>
+  </si>
+  <si>
+    <t>SAMPLE26</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1068</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1071</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1073</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1072</t>
+  </si>
+  <si>
+    <t>Crossroads Veterinary Clinic</t>
+  </si>
+  <si>
+    <t>ORD-EPL-1076</t>
+  </si>
+  <si>
+    <t>Equine Sports Medicine &amp; Surgery</t>
+  </si>
+  <si>
+    <t>FREE_VIALS</t>
+  </si>
+  <si>
+    <t>21 invoices</t>
   </si>
 </sst>
 </file>
@@ -160,7 +293,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -221,6 +354,47 @@
       <b/>
       <sz val="12"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="123F35"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="7A7974"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="DA7101"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <color rgb="964219"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="7A7974"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="DA7101"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="123F35"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0F5E4F"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="964219"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -252,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -291,6 +465,49 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1440,4 +1657,907 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L28"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="5" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" s="22" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="23">
+        <v>46113.5</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="24">
+        <v>1</v>
+      </c>
+      <c r="E6" s="12">
+        <v>1495</v>
+      </c>
+      <c r="F6" s="25">
+        <v>895</v>
+      </c>
+      <c r="G6" s="26">
+        <v>600</v>
+      </c>
+      <c r="H6" s="12">
+        <v>600</v>
+      </c>
+      <c r="I6" s="16">
+        <v>600</v>
+      </c>
+      <c r="J6" s="23">
+        <v>46119.5</v>
+      </c>
+      <c r="K6" s="27">
+        <v>0</v>
+      </c>
+      <c r="L6" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="23">
+        <v>46118.5</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="24">
+        <v>3</v>
+      </c>
+      <c r="E7" s="12">
+        <v>4485</v>
+      </c>
+      <c r="F7" s="25">
+        <v>2685</v>
+      </c>
+      <c r="G7" s="26">
+        <v>1800</v>
+      </c>
+      <c r="H7" s="12">
+        <v>1800</v>
+      </c>
+      <c r="I7" s="16">
+        <v>1800</v>
+      </c>
+      <c r="J7" s="23">
+        <v>46119.5</v>
+      </c>
+      <c r="K7" s="27">
+        <v>0</v>
+      </c>
+      <c r="L7" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="23">
+        <v>46120.5</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="24">
+        <v>1</v>
+      </c>
+      <c r="E8" s="12">
+        <v>825</v>
+      </c>
+      <c r="F8" s="25">
+        <v>475</v>
+      </c>
+      <c r="G8" s="26">
+        <v>350</v>
+      </c>
+      <c r="H8" s="12">
+        <v>350</v>
+      </c>
+      <c r="I8" s="16">
+        <v>350</v>
+      </c>
+      <c r="J8" s="23">
+        <v>46174.5</v>
+      </c>
+      <c r="K8" s="27">
+        <v>0</v>
+      </c>
+      <c r="L8" s="28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="23">
+        <v>46121.5</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="24">
+        <v>4</v>
+      </c>
+      <c r="E9" s="12">
+        <v>2400</v>
+      </c>
+      <c r="F9" s="27">
+        <v>0</v>
+      </c>
+      <c r="G9" s="26">
+        <v>2400</v>
+      </c>
+      <c r="H9" s="12">
+        <v>2400</v>
+      </c>
+      <c r="I9" s="16">
+        <v>2400</v>
+      </c>
+      <c r="J9" s="23">
+        <v>46133.5</v>
+      </c>
+      <c r="K9" s="27">
+        <v>0</v>
+      </c>
+      <c r="L9" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="23">
+        <v>46122.5</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="24">
+        <v>3</v>
+      </c>
+      <c r="E10" s="12">
+        <v>2475</v>
+      </c>
+      <c r="F10" s="25">
+        <v>675</v>
+      </c>
+      <c r="G10" s="26">
+        <v>1800</v>
+      </c>
+      <c r="H10" s="12">
+        <v>1800</v>
+      </c>
+      <c r="I10" s="16">
+        <v>1800</v>
+      </c>
+      <c r="J10" s="23">
+        <v>46154.5</v>
+      </c>
+      <c r="K10" s="27">
+        <v>0</v>
+      </c>
+      <c r="L10" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="23">
+        <v>46125.5</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="24">
+        <v>1</v>
+      </c>
+      <c r="E11" s="12">
+        <v>825</v>
+      </c>
+      <c r="F11" s="25">
+        <v>475</v>
+      </c>
+      <c r="G11" s="26">
+        <v>350</v>
+      </c>
+      <c r="H11" s="12">
+        <v>350</v>
+      </c>
+      <c r="I11" s="16">
+        <v>350</v>
+      </c>
+      <c r="J11" s="23">
+        <v>46132.5</v>
+      </c>
+      <c r="K11" s="27">
+        <v>0</v>
+      </c>
+      <c r="L11" s="28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="23">
+        <v>46125.5</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="24">
+        <v>2</v>
+      </c>
+      <c r="E12" s="12">
+        <v>1650</v>
+      </c>
+      <c r="F12" s="25">
+        <v>450</v>
+      </c>
+      <c r="G12" s="26">
+        <v>1200</v>
+      </c>
+      <c r="H12" s="12">
+        <v>1200</v>
+      </c>
+      <c r="I12" s="16">
+        <v>1200</v>
+      </c>
+      <c r="J12" s="23">
+        <v>46148.5</v>
+      </c>
+      <c r="K12" s="27">
+        <v>0</v>
+      </c>
+      <c r="L12" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="23">
+        <v>46125.5</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="24">
+        <v>2</v>
+      </c>
+      <c r="E13" s="12">
+        <v>1650</v>
+      </c>
+      <c r="F13" s="25">
+        <v>450</v>
+      </c>
+      <c r="G13" s="26">
+        <v>1200</v>
+      </c>
+      <c r="H13" s="12">
+        <v>1200</v>
+      </c>
+      <c r="I13" s="16">
+        <v>1200</v>
+      </c>
+      <c r="J13" s="23">
+        <v>46148.5</v>
+      </c>
+      <c r="K13" s="27">
+        <v>0</v>
+      </c>
+      <c r="L13" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" s="23">
+        <v>46127.5</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="24">
+        <v>1</v>
+      </c>
+      <c r="E14" s="12">
+        <v>825</v>
+      </c>
+      <c r="F14" s="25">
+        <v>225</v>
+      </c>
+      <c r="G14" s="26">
+        <v>600</v>
+      </c>
+      <c r="H14" s="12">
+        <v>600</v>
+      </c>
+      <c r="I14" s="27">
+        <v>0</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="K14" s="29">
+        <v>600</v>
+      </c>
+      <c r="L14" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="23">
+        <v>46127.5</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" s="24">
+        <v>12</v>
+      </c>
+      <c r="E15" s="12">
+        <v>9900</v>
+      </c>
+      <c r="F15" s="25">
+        <v>2700</v>
+      </c>
+      <c r="G15" s="26">
+        <v>7200</v>
+      </c>
+      <c r="H15" s="12">
+        <v>7200</v>
+      </c>
+      <c r="I15" s="16">
+        <v>7200</v>
+      </c>
+      <c r="J15" s="23">
+        <v>46188.5</v>
+      </c>
+      <c r="K15" s="27">
+        <v>0</v>
+      </c>
+      <c r="L15" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="23">
+        <v>46128.5</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="24">
+        <v>4</v>
+      </c>
+      <c r="E16" s="12">
+        <v>2400</v>
+      </c>
+      <c r="F16" s="27">
+        <v>0</v>
+      </c>
+      <c r="G16" s="26">
+        <v>2400</v>
+      </c>
+      <c r="H16" s="12">
+        <v>2400</v>
+      </c>
+      <c r="I16" s="16">
+        <v>2400</v>
+      </c>
+      <c r="J16" s="23">
+        <v>46133.5</v>
+      </c>
+      <c r="K16" s="27">
+        <v>0</v>
+      </c>
+      <c r="L16" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="23">
+        <v>46129.5</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="24">
+        <v>1</v>
+      </c>
+      <c r="E17" s="12">
+        <v>825</v>
+      </c>
+      <c r="F17" s="25">
+        <v>225</v>
+      </c>
+      <c r="G17" s="26">
+        <v>600</v>
+      </c>
+      <c r="H17" s="12">
+        <v>600</v>
+      </c>
+      <c r="I17" s="16">
+        <v>600</v>
+      </c>
+      <c r="J17" s="23">
+        <v>46133.5</v>
+      </c>
+      <c r="K17" s="27">
+        <v>0</v>
+      </c>
+      <c r="L17" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="23">
+        <v>46133.5</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" s="24">
+        <v>1</v>
+      </c>
+      <c r="E18" s="12">
+        <v>825</v>
+      </c>
+      <c r="F18" s="25">
+        <v>225</v>
+      </c>
+      <c r="G18" s="26">
+        <v>600</v>
+      </c>
+      <c r="H18" s="12">
+        <v>600</v>
+      </c>
+      <c r="I18" s="16">
+        <v>617.94</v>
+      </c>
+      <c r="J18" s="23">
+        <v>46148.5</v>
+      </c>
+      <c r="K18" s="27">
+        <v>0</v>
+      </c>
+      <c r="L18" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="23">
+        <v>46133.5</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="24">
+        <v>4</v>
+      </c>
+      <c r="E19" s="12">
+        <v>3300</v>
+      </c>
+      <c r="F19" s="25">
+        <v>900</v>
+      </c>
+      <c r="G19" s="26">
+        <v>2400</v>
+      </c>
+      <c r="H19" s="12">
+        <v>2400</v>
+      </c>
+      <c r="I19" s="16">
+        <v>2400</v>
+      </c>
+      <c r="J19" s="23">
+        <v>46143.5</v>
+      </c>
+      <c r="K19" s="27">
+        <v>0</v>
+      </c>
+      <c r="L19" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="23">
+        <v>46135.5</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" s="24">
+        <v>8</v>
+      </c>
+      <c r="E20" s="12">
+        <v>6600</v>
+      </c>
+      <c r="F20" s="25">
+        <v>1800</v>
+      </c>
+      <c r="G20" s="26">
+        <v>4800</v>
+      </c>
+      <c r="H20" s="12">
+        <v>4800</v>
+      </c>
+      <c r="I20" s="16">
+        <v>4800</v>
+      </c>
+      <c r="J20" s="23">
+        <v>46144.5</v>
+      </c>
+      <c r="K20" s="27">
+        <v>0</v>
+      </c>
+      <c r="L20" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="23">
+        <v>46135.5</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="24">
+        <v>2</v>
+      </c>
+      <c r="E21" s="12">
+        <v>1650</v>
+      </c>
+      <c r="F21" s="25">
+        <v>1650</v>
+      </c>
+      <c r="G21" s="26">
+        <v>0</v>
+      </c>
+      <c r="H21" s="12">
+        <v>0</v>
+      </c>
+      <c r="I21" s="27">
+        <v>0</v>
+      </c>
+      <c r="J21" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="K21" s="27">
+        <v>0</v>
+      </c>
+      <c r="L21" s="28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="23">
+        <v>46135.5</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" s="24">
+        <v>8</v>
+      </c>
+      <c r="E22" s="12">
+        <v>6600</v>
+      </c>
+      <c r="F22" s="25">
+        <v>1800</v>
+      </c>
+      <c r="G22" s="26">
+        <v>4800</v>
+      </c>
+      <c r="H22" s="12">
+        <v>4800</v>
+      </c>
+      <c r="I22" s="16">
+        <v>4800</v>
+      </c>
+      <c r="J22" s="23">
+        <v>46171.5</v>
+      </c>
+      <c r="K22" s="27">
+        <v>0</v>
+      </c>
+      <c r="L22" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="23">
+        <v>46139.5</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="24">
+        <v>10</v>
+      </c>
+      <c r="E23" s="12">
+        <v>8250</v>
+      </c>
+      <c r="F23" s="25">
+        <v>2250</v>
+      </c>
+      <c r="G23" s="26">
+        <v>6000</v>
+      </c>
+      <c r="H23" s="12">
+        <v>6000</v>
+      </c>
+      <c r="I23" s="16">
+        <v>6000</v>
+      </c>
+      <c r="J23" s="23">
+        <v>46148.5</v>
+      </c>
+      <c r="K23" s="27">
+        <v>0</v>
+      </c>
+      <c r="L23" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="23">
+        <v>46140.5</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="24">
+        <v>4</v>
+      </c>
+      <c r="E24" s="12">
+        <v>3300</v>
+      </c>
+      <c r="F24" s="25">
+        <v>900</v>
+      </c>
+      <c r="G24" s="26">
+        <v>2400</v>
+      </c>
+      <c r="H24" s="12">
+        <v>2400</v>
+      </c>
+      <c r="I24" s="16">
+        <v>2400</v>
+      </c>
+      <c r="J24" s="23">
+        <v>46143.5</v>
+      </c>
+      <c r="K24" s="27">
+        <v>0</v>
+      </c>
+      <c r="L24" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="23">
+        <v>46140.5</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="24">
+        <v>1</v>
+      </c>
+      <c r="E25" s="12">
+        <v>825</v>
+      </c>
+      <c r="F25" s="25">
+        <v>225</v>
+      </c>
+      <c r="G25" s="26">
+        <v>600</v>
+      </c>
+      <c r="H25" s="12">
+        <v>600</v>
+      </c>
+      <c r="I25" s="16">
+        <v>600</v>
+      </c>
+      <c r="J25" s="23">
+        <v>46153.5</v>
+      </c>
+      <c r="K25" s="27">
+        <v>0</v>
+      </c>
+      <c r="L25" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" s="23">
+        <v>46141.5</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D26" s="24">
+        <v>6</v>
+      </c>
+      <c r="E26" s="12">
+        <v>4950</v>
+      </c>
+      <c r="F26" s="25">
+        <v>4950</v>
+      </c>
+      <c r="G26" s="26">
+        <v>0</v>
+      </c>
+      <c r="H26" s="12">
+        <v>0</v>
+      </c>
+      <c r="I26" s="27">
+        <v>0</v>
+      </c>
+      <c r="J26" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="K26" s="27">
+        <v>0</v>
+      </c>
+      <c r="L26" s="28" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="32">
+        <v>79</v>
+      </c>
+      <c r="E28" s="26">
+        <v>66055</v>
+      </c>
+      <c r="F28" s="33">
+        <v>23955</v>
+      </c>
+      <c r="G28" s="34">
+        <v>42100</v>
+      </c>
+      <c r="H28" s="26">
+        <v>42100</v>
+      </c>
+      <c r="I28" s="35">
+        <v>41517.94</v>
+      </c>
+      <c r="K28" s="36">
+        <v>600</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>